<commit_message>
Add exportRequirements script and wire into buildAll
Exports each requirements/*.slreqx to a sibling xlsx with columns
Id, Summary, Description, Rationale, DerivedFrom. DerivedFrom is
populated from incoming Derive links, so parent refs live in their
own column instead of shadowing Rationale. Also produces TestCases.xlsx.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/GalacticSoup/requirements/StakeholderNeeds.xlsx
+++ b/examples/GalacticSoup/requirements/StakeholderNeeds.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="37" uniqueCount="37">
   <si>
     <t>Id</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>Facility may be deployed on any of a diverse set of worlds.</t>
+  </si>
+  <si>
+    <t>DerivedFrom</t>
   </si>
 </sst>
 </file>
@@ -166,13 +169,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.6640625" customWidth="true"/>
     <col min="2" max="2" width="21.77734375" customWidth="true"/>
     <col min="3" max="3" width="65.21875" customWidth="true"/>
     <col min="4" max="4" width="40.21875" customWidth="true"/>
+    <col min="5" max="5" width="11.44140625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -188,6 +192,9 @@
       <c r="D1" s="0" t="s">
         <v>27</v>
       </c>
+      <c r="E1" s="0" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
@@ -202,6 +209,7 @@
       <c r="D2" s="0" t="s">
         <v>28</v>
       </c>
+      <c r="E2" s="0"/>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
@@ -216,6 +224,7 @@
       <c r="D3" s="0" t="s">
         <v>29</v>
       </c>
+      <c r="E3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
@@ -230,6 +239,7 @@
       <c r="D4" s="0" t="s">
         <v>30</v>
       </c>
+      <c r="E4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
@@ -244,6 +254,7 @@
       <c r="D5" s="0" t="s">
         <v>31</v>
       </c>
+      <c r="E5" s="0"/>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
@@ -258,6 +269,7 @@
       <c r="D6" s="0" t="s">
         <v>32</v>
       </c>
+      <c r="E6" s="0"/>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
@@ -272,6 +284,7 @@
       <c r="D7" s="0" t="s">
         <v>33</v>
       </c>
+      <c r="E7" s="0"/>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
@@ -286,6 +299,7 @@
       <c r="D8" s="0" t="s">
         <v>34</v>
       </c>
+      <c r="E8" s="0"/>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
@@ -300,6 +314,7 @@
       <c r="D9" s="0" t="s">
         <v>35</v>
       </c>
+      <c r="E9" s="0"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>